<commit_message>
Add points for 57dotnff3xaafnxfltzt4czdg_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/57dotnff3xaafnxfltzt4czdg_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/57dotnff3xaafnxfltzt4czdg_playerlog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI32"/>
+  <dimension ref="A1:BI35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -790,14 +790,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -845,7 +845,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -971,14 +971,14 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -1024,21 +1024,21 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>0.73207604</v>
+        <v>0.98083557</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>+0.32</t>
+          <t>+0.53</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1164,14 +1164,14 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1217,21 +1217,21 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.61581391</v>
+        <v>0.76125</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>+0.21</t>
+          <t>+0.31</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1416,11 +1416,11 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>+0.15</t>
+          <t>+0.10</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
@@ -1552,14 +1552,14 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1605,21 +1605,21 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>1.14086367</v>
+        <v>1.21926985</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>+0.73</t>
+          <t>+0.77</t>
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL6" t="n">
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN6" t="n">
         <v>0</v>
@@ -1634,7 +1634,7 @@
         <v>0</v>
       </c>
       <c r="AR6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AS6" t="n">
         <v>4</v>
@@ -1731,10 +1731,12 @@
           <t>7fmpgkx58o9pivo2bbnxxkt05</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>3</v>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
@@ -1790,7 +1792,7 @@
         <v>0.4</v>
       </c>
       <c r="AG7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1798,15 +1800,15 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.91978319</v>
+        <v>0.87905718</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>+0.51</t>
+          <t>+0.43</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
@@ -1938,14 +1940,14 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1953,7 +1955,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -1991,11 +1993,11 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>1.53733895</v>
+        <v>1.75708656</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>+1.13</t>
+          <t>+1.30</t>
         </is>
       </c>
       <c r="AK8" t="n">
@@ -2005,7 +2007,7 @@
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN8" t="n">
         <v>0</v>
@@ -2117,10 +2119,12 @@
           <t>dqfk7czrayirrvonirtk2mk15</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
@@ -2176,7 +2180,7 @@
         <v>0.1</v>
       </c>
       <c r="AG9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
@@ -2184,15 +2188,15 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>1.13474191</v>
+        <v>1.19567343</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>+0.73</t>
+          <t>+0.74</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AL9" t="n">
         <v>0</v>
@@ -2383,11 +2387,11 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>+0.21</t>
+          <t>+0.17</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AL10" t="n">
         <v>0</v>
@@ -2578,11 +2582,11 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>+0.50</t>
+          <t>+0.46</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
@@ -2773,11 +2777,11 @@
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>+0.01</t>
+          <t>-0.03</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
@@ -2867,17 +2871,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mikel Merino</t>
+          <t>Eric García</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6</t>
+          <t xml:space="preserve"> 4</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2892,7 +2896,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>atigcsq78g14w82lwvay26aj9</t>
+          <t>4ggz7e009bq3yltc9o6mifbah</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -2902,10 +2906,10 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="L13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -2913,22 +2917,22 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="Q13" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S13" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
@@ -2958,29 +2962,29 @@
         <v>-0</v>
       </c>
       <c r="AG13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>Mikel Merino</t>
+          <t>Eric García</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>0.005370659999999985</v>
+        <v>-0.01079299</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>-0.40</t>
+          <t>-0.46</t>
         </is>
       </c>
       <c r="AK13" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="AL13" t="n">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="AM13" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -2989,13 +2993,13 @@
         <v>0</v>
       </c>
       <c r="AP13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ13" t="n">
         <v>0</v>
       </c>
       <c r="AR13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS13" t="n">
         <v>0</v>
@@ -3033,22 +3037,18 @@
       <c r="BD13" t="n">
         <v>0</v>
       </c>
-      <c r="BE13" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
+      <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BG13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BH13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BI13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -3064,17 +3064,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Ferran Torres</t>
+          <t>Mikel Merino</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7</t>
+          <t xml:space="preserve"> 6</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2szgrzcosfeifh664tgt3mfvt</t>
+          <t>atigcsq78g14w82lwvay26aj9</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -3099,7 +3099,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="L14" t="n">
         <v>2</v>
@@ -3110,22 +3110,22 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="Q14" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
@@ -3152,32 +3152,32 @@
         <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG14" t="n">
         <v>2</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>Ferran Torres</t>
+          <t>Mikel Merino</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.48235846</v>
+        <v>0.26577299</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>+0.07</t>
+          <t>-0.19</t>
         </is>
       </c>
       <c r="AK14" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="AL14" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="AM14" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3186,13 +3186,13 @@
         <v>0</v>
       </c>
       <c r="AP14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ14" t="n">
         <v>0</v>
       </c>
       <c r="AR14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS14" t="n">
         <v>0</v>
@@ -3207,7 +3207,7 @@
         <v>0</v>
       </c>
       <c r="AW14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX14" t="n">
         <v>0</v>
@@ -3232,11 +3232,11 @@
       </c>
       <c r="BE14" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="BF14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG14" t="n">
         <v>1</v>
@@ -3261,17 +3261,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Nico Williams</t>
+          <t>Ferran Torres</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 17</t>
+          <t xml:space="preserve"> 7</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>66jotyvbhtz5cjvhbby6luelm</t>
+          <t>2szgrzcosfeifh664tgt3mfvt</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -3296,7 +3296,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="L15" t="n">
         <v>2</v>
@@ -3307,22 +3307,22 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="Q15" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S15" t="n">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
@@ -3356,25 +3356,25 @@
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>Nico Williams</t>
+          <t>Ferran Torres</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0.36066287</v>
+        <v>0.57168269</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>-0.05</t>
+          <t>+0.12</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="AL15" t="n">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="AM15" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3386,7 +3386,7 @@
         <v>0</v>
       </c>
       <c r="AQ15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR15" t="n">
         <v>0</v>
@@ -3395,7 +3395,7 @@
         <v>0</v>
       </c>
       <c r="AT15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU15" t="n">
         <v>0</v>
@@ -3433,10 +3433,10 @@
         </is>
       </c>
       <c r="BF15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BG15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BH15" t="n">
         <v>1</v>
@@ -3458,17 +3458,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pedri</t>
+          <t>Nico Williams</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 20</t>
+          <t xml:space="preserve"> 17</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LW</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>4ftlhtels58lyzfluwofzwxuy</t>
+          <t>66jotyvbhtz5cjvhbby6luelm</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -3493,7 +3493,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="L16" t="n">
         <v>2</v>
@@ -3504,22 +3504,22 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="Q16" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LW</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -3546,32 +3546,32 @@
         <v>0</v>
       </c>
       <c r="AF16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AG16" t="n">
         <v>2</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Pedri</t>
+          <t>Nico Williams</t>
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.6438842600000001</v>
+        <v>0.9422833999999999</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>+0.24</t>
+          <t>+0.49</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AL16" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="AM16" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3580,28 +3580,28 @@
         <v>0</v>
       </c>
       <c r="AP16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV16" t="n">
         <v>0</v>
       </c>
       <c r="AW16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AX16" t="n">
         <v>0</v>
@@ -3626,14 +3626,14 @@
       </c>
       <c r="BE16" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>FWD</t>
         </is>
       </c>
       <c r="BF16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG16" t="n">
         <v>5</v>
-      </c>
-      <c r="BG16" t="n">
-        <v>2</v>
       </c>
       <c r="BH16" t="n">
         <v>1</v>
@@ -3650,37 +3650,37 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+          <t>eh7yt2x2wck51oixw8012ux5j</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>E. Martínez</t>
+          <t>Martín Zubimendi</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>23</t>
+          <t xml:space="preserve"> 18</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>3zl1q2gk6tdmzirsyfgm38no5</t>
+          <t>80aqmv4ht6rs1812qrr5j8kix</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -3689,30 +3689,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>98</v>
+      </c>
+      <c r="L17" t="n">
+        <v>3</v>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>98</v>
+        <v>4</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="Q17" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>98</v>
+        <v>4</v>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -3724,12 +3728,12 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+          <t>eh7yt2x2wck51oixw8012ux5j</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="AD17" t="n">
@@ -3739,20 +3743,32 @@
         <v>0</v>
       </c>
       <c r="AF17" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH17" t="inlineStr"/>
-      <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>Martín Zubimendi</t>
+        </is>
+      </c>
+      <c r="AI17" t="n">
+        <v>0.0597685</v>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>-0.39</t>
+        </is>
+      </c>
+      <c r="AK17" t="n">
+        <v>24</v>
+      </c>
       <c r="AL17" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="AM17" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3767,10 +3783,10 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT17" t="n">
         <v>0</v>
@@ -3779,7 +3795,7 @@
         <v>0</v>
       </c>
       <c r="AV17" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -3805,11 +3821,7 @@
       <c r="BD17" t="n">
         <v>0</v>
       </c>
-      <c r="BE17" t="inlineStr">
-        <is>
-          <t>GK</t>
-        </is>
-      </c>
+      <c r="BE17" t="inlineStr"/>
       <c r="BF17" t="n">
         <v>0</v>
       </c>
@@ -3817,10 +3829,10 @@
         <v>0</v>
       </c>
       <c r="BH17" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="BI17" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3831,71 +3843,73 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+          <t>eh7yt2x2wck51oixw8012ux5j</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>G. Montiel</t>
+          <t>Pedri</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 4</t>
+          <t xml:space="preserve"> 20</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>4ftlhtels58lyzfluwofzwxuy</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>61</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>1y74tse0vpdxanxf152cc8jjd</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>2</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="N18" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="Q18" t="n">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="S18" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3907,12 +3921,12 @@
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+          <t>eh7yt2x2wck51oixw8012ux5j</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="AD18" t="n">
@@ -3929,25 +3943,25 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>G. Montiel</t>
+          <t>Pedri</t>
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>0.33622127</v>
+        <v>1.30041563</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>+0.85</t>
         </is>
       </c>
       <c r="AK18" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="AL18" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="AM18" t="n">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
@@ -3956,19 +3970,19 @@
         <v>0</v>
       </c>
       <c r="AP18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AQ18" t="n">
         <v>0</v>
       </c>
       <c r="AR18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AS18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AT18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU18" t="n">
         <v>1</v>
@@ -3977,7 +3991,7 @@
         <v>0</v>
       </c>
       <c r="AW18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX18" t="n">
         <v>0</v>
@@ -4000,18 +4014,22 @@
       <c r="BD18" t="n">
         <v>0</v>
       </c>
-      <c r="BE18" t="inlineStr"/>
+      <c r="BE18" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
       <c r="BF18" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="BG18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BH18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BI18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -4027,17 +4045,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>N. Tagliafico</t>
+          <t>E. Martínez</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 3</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -4047,12 +4065,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>40hu79d2a4k94nc52z7dblpsl</t>
+          <t>3zl1q2gk6tdmzirsyfgm38no5</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -4069,22 +4087,22 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -4111,32 +4129,20 @@
         <v>0</v>
       </c>
       <c r="AF19" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="AG19" t="n">
         <v>1</v>
       </c>
-      <c r="AH19" t="inlineStr">
-        <is>
-          <t>N. Tagliafico</t>
-        </is>
-      </c>
-      <c r="AI19" t="n">
-        <v>0.62600681</v>
-      </c>
-      <c r="AJ19" t="inlineStr">
-        <is>
-          <t>+0.22</t>
-        </is>
-      </c>
-      <c r="AK19" t="n">
-        <v>9</v>
-      </c>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr"/>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
@@ -4148,22 +4154,22 @@
         <v>0</v>
       </c>
       <c r="AQ19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AS19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AT19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AU19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV19" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AW19" t="n">
         <v>0</v>
@@ -4191,20 +4197,20 @@
       </c>
       <c r="BE19" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="BF19" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="BG19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BH19" t="n">
-        <v>6</v>
+        <v>11.5</v>
       </c>
       <c r="BI19" t="n">
-        <v>6</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="20">
@@ -4220,17 +4226,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>E. Fernández</t>
+          <t>G. Montiel</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 24</t>
+          <t xml:space="preserve"> 4</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4240,18 +4246,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1zxwich342p8fholev7ddkwh6</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
+          <t>1y74tse0vpdxanxf152cc8jjd</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>2</v>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -4262,35 +4270,25 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>92</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>CM(3)</t>
-        </is>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>45</v>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>CM(3)</t>
-        </is>
-      </c>
-      <c r="U20" t="n">
-        <v>47</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
@@ -4314,32 +4312,32 @@
         <v>0</v>
       </c>
       <c r="AF20" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="AG20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>E. Fernández</t>
+          <t>G. Montiel</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>-0.69539225</v>
+        <v>0.33622127</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>-1.10</t>
+          <t>-0.12</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="AL20" t="n">
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="AN20" t="n">
         <v>0</v>
@@ -4351,13 +4349,13 @@
         <v>0</v>
       </c>
       <c r="AQ20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR20" t="n">
         <v>2</v>
       </c>
       <c r="AS20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT20" t="n">
         <v>2</v>
@@ -4366,16 +4364,16 @@
         <v>1</v>
       </c>
       <c r="AV20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW20" t="n">
         <v>0</v>
       </c>
       <c r="AX20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AZ20" t="n">
         <v>0</v>
@@ -4392,16 +4390,12 @@
       <c r="BD20" t="n">
         <v>0</v>
       </c>
-      <c r="BE20" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
+      <c r="BE20" t="inlineStr"/>
       <c r="BF20" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="BG20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BH20" t="n">
         <v>0</v>
@@ -4423,17 +4417,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C. Romero</t>
+          <t>N. Tagliafico</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 13</t>
+          <t xml:space="preserve"> 3</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4443,20 +4437,18 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2w7i4jfw5wgh3j2wuworoumeh</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>2</v>
-      </c>
+          <t>40hu79d2a4k94nc52z7dblpsl</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -4467,25 +4459,35 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>69</v>
-      </c>
-      <c r="O21" t="inlineStr"/>
+        <v>102</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>69</v>
-      </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
+        <v>101.3</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="U21" t="n">
+        <v>0.7</v>
+      </c>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
@@ -4512,29 +4514,29 @@
         <v>0.4</v>
       </c>
       <c r="AG21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>C. Romero</t>
+          <t>N. Tagliafico</t>
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.12852338</v>
+        <v>0.70351055</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>-0.28</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="AL21" t="n">
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="AN21" t="n">
         <v>0</v>
@@ -4546,19 +4548,19 @@
         <v>0</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR21" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS21" t="n">
         <v>3</v>
       </c>
-      <c r="AS21" t="n">
-        <v>1</v>
-      </c>
       <c r="AT21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AU21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AV21" t="n">
         <v>0</v>
@@ -4567,7 +4569,7 @@
         <v>0</v>
       </c>
       <c r="AX21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY21" t="n">
         <v>0</v>
@@ -4593,16 +4595,16 @@
         </is>
       </c>
       <c r="BF21" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="BG21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BI21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -4618,17 +4620,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Lisandro Martínez</t>
+          <t>E. Fernández</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6</t>
+          <t xml:space="preserve"> 24</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4638,20 +4640,18 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>b17tkj4ea4jld8yupekcolall</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>1</v>
-      </c>
+          <t>1zxwich342p8fholev7ddkwh6</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
@@ -4662,25 +4662,35 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>43</v>
-      </c>
-      <c r="O22" t="inlineStr"/>
+        <v>92</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>CM(3)</t>
+        </is>
+      </c>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="S22" t="n">
-        <v>43</v>
-      </c>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
+        <v>45</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>CM(3)</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>47</v>
+      </c>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
@@ -4704,32 +4714,32 @@
         <v>0</v>
       </c>
       <c r="AF22" t="n">
-        <v>-0</v>
+        <v>0.1</v>
       </c>
       <c r="AG22" t="n">
         <v>1</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>Lisandro Martínez</t>
+          <t>E. Fernández</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.18245016</v>
+        <v>-0.69539225</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-1.15</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -4741,22 +4751,22 @@
         <v>0</v>
       </c>
       <c r="AQ22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AR22" t="n">
         <v>2</v>
       </c>
       <c r="AS22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AT22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU22" t="n">
         <v>1</v>
       </c>
       <c r="AV22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW22" t="n">
         <v>0</v>
@@ -4765,7 +4775,7 @@
         <v>1</v>
       </c>
       <c r="AY22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AZ22" t="n">
         <v>0</v>
@@ -4784,14 +4794,14 @@
       </c>
       <c r="BE22" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="BF22" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="BG22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BH22" t="n">
         <v>0</v>
@@ -4813,17 +4823,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>R. De Paul</t>
+          <t>C. Romero</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7</t>
+          <t xml:space="preserve"> 13</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4833,12 +4843,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>3ga7qj3h3dbmqucxmaxhmrjdh</t>
+          <t>2w7i4jfw5wgh3j2wuworoumeh</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -4859,11 +4869,7 @@
       <c r="N23" t="n">
         <v>69</v>
       </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>RCM(3)</t>
-        </is>
-      </c>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
@@ -4872,20 +4878,14 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="S23" t="n">
-        <v>45</v>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>RCM(3)</t>
-        </is>
-      </c>
-      <c r="U23" t="n">
-        <v>24</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
@@ -4909,26 +4909,26 @@
         <v>0</v>
       </c>
       <c r="AF23" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="AG23" t="n">
         <v>2</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>R. De Paul</t>
+          <t>C. Romero</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>-0.01371803000000002</v>
+        <v>0.12852338</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>-0.42</t>
+          <t>-0.33</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
@@ -4958,7 +4958,7 @@
         <v>0</v>
       </c>
       <c r="AU23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV23" t="n">
         <v>0</v>
@@ -4967,7 +4967,7 @@
         <v>0</v>
       </c>
       <c r="AX23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY23" t="n">
         <v>0</v>
@@ -4989,20 +4989,20 @@
       </c>
       <c r="BE23" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="BF23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BG23" t="n">
         <v>0</v>
       </c>
       <c r="BH23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BI23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
@@ -5018,17 +5018,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A. Mac Allister</t>
+          <t>Lisandro Martínez</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 20</t>
+          <t xml:space="preserve"> 6</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -5038,18 +5038,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>am6ppbdrbz4ml3xsbty53o73d</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>b17tkj4ea4jld8yupekcolall</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -5060,35 +5062,25 @@
         </is>
       </c>
       <c r="N24" t="n">
-        <v>98</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>LCM(3)</t>
-        </is>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>98</v>
+        <v>43</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S24" t="n">
-        <v>45</v>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>LCM(3)</t>
-        </is>
-      </c>
-      <c r="U24" t="n">
-        <v>53</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
@@ -5112,32 +5104,32 @@
         <v>0</v>
       </c>
       <c r="AF24" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="AG24" t="n">
         <v>1</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
-          <t>A. Mac Allister</t>
+          <t>Lisandro Martínez</t>
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>0.5206167900000001</v>
+        <v>0.18245016</v>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>+0.11</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="AK24" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="AL24" t="n">
         <v>0</v>
       </c>
       <c r="AM24" t="n">
-        <v>98</v>
+        <v>43</v>
       </c>
       <c r="AN24" t="n">
         <v>0</v>
@@ -5149,10 +5141,10 @@
         <v>0</v>
       </c>
       <c r="AQ24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AS24" t="n">
         <v>2</v>
@@ -5161,7 +5153,7 @@
         <v>1</v>
       </c>
       <c r="AU24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AV24" t="n">
         <v>0</v>
@@ -5170,7 +5162,7 @@
         <v>0</v>
       </c>
       <c r="AX24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY24" t="n">
         <v>0</v>
@@ -5192,20 +5184,20 @@
       </c>
       <c r="BE24" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="BF24" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="BG24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BH24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BI24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -5221,17 +5213,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>J. Alvarez</t>
+          <t>R. De Paul</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 9</t>
+          <t xml:space="preserve"> 7</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RM</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -5241,18 +5233,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>9ikkuxd19avliz1khcrm82gyy</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
+          <t>3ga7qj3h3dbmqucxmaxhmrjdh</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>2</v>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -5263,22 +5257,22 @@
         </is>
       </c>
       <c r="N25" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>AM, LCF(2)</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="P25" t="n">
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RM</t>
         </is>
       </c>
       <c r="S25" t="n">
@@ -5286,20 +5280,14 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>LCF(2)</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="U25" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>AM</t>
-        </is>
-      </c>
-      <c r="W25" t="n">
-        <v>5.5</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
@@ -5321,32 +5309,32 @@
         <v>0</v>
       </c>
       <c r="AF25" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AG25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>J. Alvarez</t>
+          <t>R. De Paul</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>0.03626574</v>
+        <v>-0.01371803000000002</v>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>-0.37</t>
+          <t>-0.47</t>
         </is>
       </c>
       <c r="AK25" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="AL25" t="n">
         <v>0</v>
       </c>
       <c r="AM25" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="AN25" t="n">
         <v>0</v>
@@ -5358,19 +5346,19 @@
         <v>0</v>
       </c>
       <c r="AQ25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR25" t="n">
         <v>3</v>
       </c>
       <c r="AS25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV25" t="n">
         <v>0</v>
@@ -5401,20 +5389,20 @@
       </c>
       <c r="BE25" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="BF25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BG25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BH25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BI25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
@@ -5430,17 +5418,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>L. Messi</t>
+          <t>A. Mac Allister</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10</t>
+          <t xml:space="preserve"> 20</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -5450,12 +5438,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>c5ryhn04g9goikd0blmh83aol</t>
+          <t>am6ppbdrbz4ml3xsbty53o73d</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -5472,22 +5460,22 @@
         </is>
       </c>
       <c r="N26" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>RCF(2)</t>
+          <t>LCM(3)</t>
         </is>
       </c>
       <c r="P26" t="n">
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="S26" t="n">
@@ -5495,11 +5483,11 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>RCF(2)</t>
+          <t>LCM(3)</t>
         </is>
       </c>
       <c r="U26" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr"/>
@@ -5524,32 +5512,32 @@
         <v>0</v>
       </c>
       <c r="AF26" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AG26" t="n">
         <v>1</v>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>L. Messi</t>
+          <t>A. Mac Allister</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>0.03950882999999999</v>
+        <v>0.5208359300000001</v>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
-          <t>-0.37</t>
+          <t>+0.07</t>
         </is>
       </c>
       <c r="AK26" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="AL26" t="n">
         <v>0</v>
       </c>
       <c r="AM26" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN26" t="n">
         <v>0</v>
@@ -5564,16 +5552,16 @@
         <v>1</v>
       </c>
       <c r="AR26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV26" t="n">
         <v>0</v>
@@ -5604,20 +5592,20 @@
       </c>
       <c r="BE26" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="BF26" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BG26" t="n">
         <v>1</v>
       </c>
       <c r="BH26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BI26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -5633,17 +5621,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>N. González</t>
+          <t>J. Alvarez</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 15</t>
+          <t xml:space="preserve"> 9</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>LM</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -5653,16 +5641,16 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>eh1ul4duphy1iz4odwx9tkjjd</t>
+          <t>9ikkuxd19avliz1khcrm82gyy</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -5677,27 +5665,43 @@
         </is>
       </c>
       <c r="N27" t="n">
-        <v>45</v>
-      </c>
-      <c r="O27" t="inlineStr"/>
+        <v>101</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>AM, LCF(2)</t>
+        </is>
+      </c>
       <c r="P27" t="n">
         <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>45</v>
+        <v>101</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>LM</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S27" t="n">
         <v>45</v>
       </c>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>LCF(2)</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="W27" t="n">
+        <v>8.5</v>
+      </c>
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
@@ -5719,32 +5723,32 @@
         <v>0</v>
       </c>
       <c r="AF27" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AG27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>N. González</t>
+          <t>J. Alvarez</t>
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>-0.02617547999999999</v>
+        <v>0.07609744</v>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
-          <t>-0.43</t>
+          <t>-0.38</t>
         </is>
       </c>
       <c r="AK27" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="AL27" t="n">
         <v>0</v>
       </c>
       <c r="AM27" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="AN27" t="n">
         <v>0</v>
@@ -5756,19 +5760,19 @@
         <v>0</v>
       </c>
       <c r="AQ27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR27" t="n">
         <v>3</v>
       </c>
       <c r="AS27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV27" t="n">
         <v>0</v>
@@ -5797,18 +5801,22 @@
       <c r="BD27" t="n">
         <v>0</v>
       </c>
-      <c r="BE27" t="inlineStr"/>
+      <c r="BE27" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
       <c r="BF27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BG27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BH27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BI27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -5824,32 +5832,32 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>L. Paredes</t>
+          <t>L. Messi</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 5</t>
+          <t xml:space="preserve"> 10</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>DM</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>apdtqouzo9b02ozdxk8mx4zbp</t>
+          <t>c5ryhn04g9goikd0blmh83aol</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -5858,46 +5866,42 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K28" t="n">
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>102</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>RCF(2)</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>102</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
         <v>45</v>
       </c>
-      <c r="L28" t="n">
-        <v>2</v>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="N28" t="n">
-        <v>53</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>RCM(2)</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>45</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>98</v>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="S28" t="n">
-        <v>47.5</v>
-      </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>RCF(2)</t>
         </is>
       </c>
       <c r="U28" t="n">
-        <v>5.5</v>
+        <v>57</v>
       </c>
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
@@ -5922,32 +5926,32 @@
         <v>0</v>
       </c>
       <c r="AF28" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AG28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>L. Paredes</t>
+          <t>L. Messi</t>
         </is>
       </c>
       <c r="AI28" t="n">
-        <v>-0.06761122000000003</v>
+        <v>0.06887319</v>
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
-          <t>-0.48</t>
+          <t>-0.39</t>
         </is>
       </c>
       <c r="AK28" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="AL28" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="AM28" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN28" t="n">
         <v>0</v>
@@ -5959,19 +5963,19 @@
         <v>0</v>
       </c>
       <c r="AQ28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR28" t="n">
         <v>1</v>
       </c>
       <c r="AS28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AT28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV28" t="n">
         <v>0</v>
@@ -5980,7 +5984,7 @@
         <v>0</v>
       </c>
       <c r="AX28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY28" t="n">
         <v>0</v>
@@ -6000,18 +6004,22 @@
       <c r="BD28" t="n">
         <v>0</v>
       </c>
-      <c r="BE28" t="inlineStr"/>
+      <c r="BE28" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
       <c r="BF28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BI28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -6027,81 +6035,69 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>G. Simeone</t>
+          <t>N. González</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 17</t>
+          <t xml:space="preserve"> 15</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>LM</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>eh1ul4duphy1iz4odwx9tkjjd</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>2</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>5es43b4a7fv0lkmp63dj439ey</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K29" t="n">
-        <v>69</v>
-      </c>
-      <c r="L29" t="n">
-        <v>2</v>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="N29" t="n">
-        <v>29</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>RCM(3)</t>
-        </is>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
       <c r="P29" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="Q29" t="n">
-        <v>98</v>
+        <v>45</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>LM</t>
         </is>
       </c>
       <c r="S29" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>RCM(3)</t>
-        </is>
-      </c>
-      <c r="U29" t="n">
-        <v>28.2</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
@@ -6132,25 +6128,25 @@
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>G. Simeone</t>
+          <t>N. González</t>
         </is>
       </c>
       <c r="AI29" t="n">
-        <v>0.08145062000000002</v>
+        <v>-0.02617547999999999</v>
       </c>
       <c r="AJ29" t="inlineStr">
         <is>
-          <t>-0.33</t>
+          <t>-0.48</t>
         </is>
       </c>
       <c r="AK29" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="AL29" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="AM29" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AN29" t="n">
         <v>0</v>
@@ -6162,10 +6158,10 @@
         <v>0</v>
       </c>
       <c r="AQ29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AR29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS29" t="n">
         <v>0</v>
@@ -6208,7 +6204,7 @@
         <v>0</v>
       </c>
       <c r="BG29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BH29" t="n">
         <v>0</v>
@@ -6230,17 +6226,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>N. Otamendi</t>
+          <t>M. Senesi</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 19</t>
+          <t xml:space="preserve"> 2</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -6255,7 +6251,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>x32fbvwwxkda9ruezw67b3dh</t>
+          <t>95pzsjfh0wf6isp6qpf9lddyh</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -6265,10 +6261,10 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -6276,34 +6272,34 @@
         </is>
       </c>
       <c r="N30" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="Q30" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S30" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
           <t>LCB(2)</t>
         </is>
       </c>
-      <c r="S30" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>RCB(2)</t>
-        </is>
-      </c>
       <c r="U30" t="n">
-        <v>28.2</v>
+        <v>0.7</v>
       </c>
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
@@ -6328,32 +6324,32 @@
         <v>0</v>
       </c>
       <c r="AF30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AG30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>N. Otamendi</t>
+          <t>M. Senesi</t>
         </is>
       </c>
       <c r="AI30" t="n">
-        <v>0.06222646999999999</v>
+        <v>0</v>
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
-          <t>-0.35</t>
+          <t>-0.45</t>
         </is>
       </c>
       <c r="AK30" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="AL30" t="n">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="AM30" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN30" t="n">
         <v>0</v>
@@ -6371,10 +6367,10 @@
         <v>0</v>
       </c>
       <c r="AS30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU30" t="n">
         <v>0</v>
@@ -6433,17 +6429,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>F. Medina</t>
+          <t>L. Paredes</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 25</t>
+          <t xml:space="preserve"> 5</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -6458,7 +6454,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>br7zigajqee6fms35zhm1sb8p</t>
+          <t>apdtqouzo9b02ozdxk8mx4zbp</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -6468,7 +6464,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="L31" t="n">
         <v>2</v>
@@ -6479,34 +6475,34 @@
         </is>
       </c>
       <c r="N31" t="n">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="Q31" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="S31" t="n">
-        <v>0.8</v>
+        <v>47.5</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="U31" t="n">
-        <v>28.2</v>
+        <v>9.5</v>
       </c>
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
@@ -6538,25 +6534,25 @@
       </c>
       <c r="AH31" t="inlineStr">
         <is>
-          <t>F. Medina</t>
+          <t>L. Paredes</t>
         </is>
       </c>
       <c r="AI31" t="n">
-        <v>0.8175034</v>
+        <v>-0.14419448</v>
       </c>
       <c r="AJ31" t="inlineStr">
         <is>
-          <t>+0.41</t>
+          <t>-0.60</t>
         </is>
       </c>
       <c r="AK31" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="AL31" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="AM31" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AN31" t="n">
         <v>0</v>
@@ -6574,13 +6570,13 @@
         <v>1</v>
       </c>
       <c r="AS31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV31" t="n">
         <v>0</v>
@@ -6589,7 +6585,7 @@
         <v>0</v>
       </c>
       <c r="AX31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY31" t="n">
         <v>0</v>
@@ -6609,22 +6605,18 @@
       <c r="BD31" t="n">
         <v>0</v>
       </c>
-      <c r="BE31" t="inlineStr">
-        <is>
-          <t>DEF</t>
-        </is>
-      </c>
+      <c r="BE31" t="inlineStr"/>
       <c r="BF31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BG31" t="n">
         <v>0</v>
       </c>
       <c r="BH31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BI31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -6640,17 +6632,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>N. Molina</t>
+          <t>G. Simeone</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 26</t>
+          <t xml:space="preserve"> 17</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>RM</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -6665,7 +6657,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>ieu0x9fy8hpqyztdjg8bgpnt</t>
+          <t>5es43b4a7fv0lkmp63dj439ey</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -6675,7 +6667,7 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="L32" t="n">
         <v>2</v>
@@ -6686,25 +6678,35 @@
         </is>
       </c>
       <c r="N32" t="n">
-        <v>41</v>
-      </c>
-      <c r="O32" t="inlineStr"/>
+        <v>33</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>RCM(3)</t>
+        </is>
+      </c>
       <c r="P32" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="Q32" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>RM</t>
         </is>
       </c>
       <c r="S32" t="n">
-        <v>41</v>
-      </c>
-      <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
+        <v>0.8</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>RCM(3)</t>
+        </is>
+      </c>
+      <c r="U32" t="n">
+        <v>32.2</v>
+      </c>
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
@@ -6735,92 +6737,701 @@
       </c>
       <c r="AH32" t="inlineStr">
         <is>
+          <t>G. Simeone</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>-0.07110935999999998</v>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>-0.53</t>
+        </is>
+      </c>
+      <c r="AK32" t="n">
+        <v>30</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>69</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>102</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE32" t="inlineStr"/>
+      <c r="BF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG32" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>57dotnff3xaafnxfltzt4czdg</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>N. Otamendi</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 19</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LCB(2)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>x32fbvwwxkda9ruezw67b3dh</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>43</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>59</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>RCB(2)</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>43</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>102</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>LCB(2)</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>RCB(2)</t>
+        </is>
+      </c>
+      <c r="U33" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="AD33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>N. Otamendi</t>
+        </is>
+      </c>
+      <c r="AI33" t="n">
+        <v>0.31968009</v>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>-0.13</t>
+        </is>
+      </c>
+      <c r="AK33" t="n">
+        <v>18</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>43</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>102</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE33" t="inlineStr"/>
+      <c r="BF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>57dotnff3xaafnxfltzt4czdg</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>F. Medina</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 25</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>RCB(2)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>br7zigajqee6fms35zhm1sb8p</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>69</v>
+      </c>
+      <c r="L34" t="n">
+        <v>2</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>33</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>LB, LCB(2)</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>69</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>102</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>RCB(2)</t>
+        </is>
+      </c>
+      <c r="S34" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>LCB(2)</t>
+        </is>
+      </c>
+      <c r="U34" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="W34" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="AD34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>F. Medina</t>
+        </is>
+      </c>
+      <c r="AI34" t="n">
+        <v>0.80741017</v>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>+0.35</t>
+        </is>
+      </c>
+      <c r="AK34" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL34" t="n">
+        <v>69</v>
+      </c>
+      <c r="AM34" t="n">
+        <v>102</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE34" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="BF34" t="n">
+        <v>4</v>
+      </c>
+      <c r="BG34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH34" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>57dotnff3xaafnxfltzt4czdg</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
           <t>N. Molina</t>
         </is>
       </c>
-      <c r="AI32" t="n">
-        <v>-0.25754083</v>
-      </c>
-      <c r="AJ32" t="inlineStr">
-        <is>
-          <t>-0.67</t>
-        </is>
-      </c>
-      <c r="AK32" t="n">
-        <v>28</v>
-      </c>
-      <c r="AL32" t="n">
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>ieu0x9fy8hpqyztdjg8bgpnt</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
         <v>57</v>
       </c>
-      <c r="AM32" t="n">
-        <v>98</v>
-      </c>
-      <c r="AN32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR32" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS32" t="n">
-        <v>2</v>
-      </c>
-      <c r="AT32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU32" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV32" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ32" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA32" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB32" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC32" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD32" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE32" t="inlineStr">
+      <c r="L35" t="n">
+        <v>2</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>45</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="n">
+        <v>57</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>102</v>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="S35" t="n">
+        <v>45</v>
+      </c>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>ak48fkypnql8y4n69cvcq5ghc</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="AD35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>N. Molina</t>
+        </is>
+      </c>
+      <c r="AI35" t="n">
+        <v>0.05603976</v>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>-0.40</t>
+        </is>
+      </c>
+      <c r="AK35" t="n">
+        <v>25</v>
+      </c>
+      <c r="AL35" t="n">
+        <v>57</v>
+      </c>
+      <c r="AM35" t="n">
+        <v>102</v>
+      </c>
+      <c r="AN35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR35" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS35" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU35" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE35" t="inlineStr">
         <is>
           <t>DEF</t>
         </is>
       </c>
-      <c r="BF32" t="n">
-        <v>5</v>
-      </c>
-      <c r="BG32" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH32" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI32" t="n">
+      <c r="BF35" t="n">
+        <v>6</v>
+      </c>
+      <c r="BG35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI35" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>